<commit_message>
fix: update washing machine price and link labels
</commit_message>
<xml_diff>
--- a/Moving out sale.xlsx
+++ b/Moving out sale.xlsx
@@ -834,7 +834,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -978,8 +978,8 @@
       <c r="B14" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>24</v>
+      <c r="C14" s="5">
+        <v>200</v>
       </c>
     </row>
     <row r="15">
@@ -1290,24 +1290,24 @@
     <mergeCell ref="A38:C38"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B3"/>
-    <hyperlink r:id="rId2" ref="B6"/>
-    <hyperlink r:id="rId3" ref="B7"/>
-    <hyperlink r:id="rId4" ref="B11"/>
-    <hyperlink r:id="rId5" ref="B12"/>
-    <hyperlink r:id="rId6" ref="B14"/>
-    <hyperlink r:id="rId7" ref="B18"/>
-    <hyperlink r:id="rId8" ref="B21"/>
-    <hyperlink r:id="rId9" ref="B22"/>
-    <hyperlink r:id="rId10" ref="B23"/>
-    <hyperlink r:id="rId11" ref="B24"/>
-    <hyperlink r:id="rId12" ref="B26"/>
-    <hyperlink r:id="rId13" ref="A28"/>
-    <hyperlink r:id="rId14" ref="B28"/>
-    <hyperlink r:id="rId15" ref="A29"/>
-    <hyperlink r:id="rId16" ref="B29"/>
-    <hyperlink r:id="rId17" ref="B30"/>
+    <hyperlink ns1:id="rId1" ref="B3"/>
+    <hyperlink ns1:id="rId2" ref="B6"/>
+    <hyperlink ns1:id="rId3" ref="B7"/>
+    <hyperlink ns1:id="rId4" ref="B11"/>
+    <hyperlink ns1:id="rId5" ref="B12"/>
+    <hyperlink ns1:id="rId6" ref="B14"/>
+    <hyperlink ns1:id="rId7" ref="B18"/>
+    <hyperlink ns1:id="rId8" ref="B21"/>
+    <hyperlink ns1:id="rId9" ref="B22"/>
+    <hyperlink ns1:id="rId10" ref="B23"/>
+    <hyperlink ns1:id="rId11" ref="B24"/>
+    <hyperlink ns1:id="rId12" ref="B26"/>
+    <hyperlink ns1:id="rId13" ref="A28"/>
+    <hyperlink ns1:id="rId14" ref="B28"/>
+    <hyperlink ns1:id="rId15" ref="A29"/>
+    <hyperlink ns1:id="rId16" ref="B29"/>
+    <hyperlink ns1:id="rId17" ref="B30"/>
   </hyperlinks>
-  <drawing r:id="rId18"/>
+  <drawing ns1:id="rId18"/>
 </worksheet>
 </file>
</xml_diff>